<commit_message>
Add jerome's annotated xlsx
</commit_message>
<xml_diff>
--- a/data_nlpforsocialinteractions/MFRC_nlpforsocialinteractions_filtered_50_jerome.xlsx
+++ b/data_nlpforsocialinteractions/MFRC_nlpforsocialinteractions_filtered_50_jerome.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
   <si>
     <t>ID</t>
   </si>
@@ -132,6 +132,9 @@
     <t xml:space="preserve">FFS its' a FRENCH election. Melenchon (19% votes didn't call to vote for him). Fillon and Hamon did but called him a lesser evil compared to a potential disaster,not exactly awe inspiring for their voters.</t>
   </si>
   <si>
+    <t xml:space="preserve">claims about authority figures</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fuck populism and people who don't understand evidence-based policy and just try to appeal to people's fears/lack of education. Fuck Trump, Fuck Bernie, Fuck Le Pen, fuck em all.</t>
   </si>
   <si>
@@ -141,118 +144,232 @@
     <t xml:space="preserve">I am for Macron but it have nothing to do with penis size. Penis size don't control the personality so let's stop shaming smaller people like me who support Macron, stop lumping me in with Trump supporters because of my size when I actually hate trump.</t>
   </si>
   <si>
+    <t xml:space="preserve">claim is about discrimination against "smaller people" which doesn't fall neatly into any</t>
+  </si>
+  <si>
     <t xml:space="preserve">I mean, you committed a crime you idiot, isnt there enough porn for you weirdos?</t>
   </si>
   <si>
+    <t xml:space="preserve">concern about sexual crime related to porn</t>
+  </si>
+  <si>
     <t xml:space="preserve">I remember working there for a month. I made $225 a week BEFORE taxes. A whopping $13k a year with NO BENEFITS. Needless to say I quit without notice on a Friday night and found a much better job. "We're all a family" Fuck off with that obvious propaganda bullshit and your starvation wages. Shit company.</t>
   </si>
   <si>
+    <t xml:space="preserve">lack of care by employer</t>
+  </si>
+  <si>
     <t xml:space="preserve">I second that. The last piece "To claim that we need to continue to exploit these broken people beyond that is just selfish and cruel...". Very good point, people are bred like cattle to provide income for the state. Disgusting!</t>
   </si>
   <si>
+    <t xml:space="preserve">exploitation, hints of disgust and corruptuon of the state</t>
+  </si>
+  <si>
     <t xml:space="preserve">I think you mistake what I mean by ruin their life, and missed an inferred exaggeration. Expose them, get them fired. Not harm them physically. Nothing that would put me in any legal or professional harm, but expose them to others which would have a negative repercussion on their life...as it well should in my opinion. They operate on a different spectrum of morals or lack there of, and are deserving of exposure, punishment and social exile. Its also not anger at the thought...its utter disgust.</t>
   </si>
   <si>
+    <t xml:space="preserve">excluding a group from society to keep it pure</t>
+  </si>
+  <si>
     <t xml:space="preserve">I would agree for any other candidate than Le Pen. For a party full of nazis, founded by nazis, with very nazi ideas, i truly think she does not represent democracy. It's not the same thing at all, and it's a valid dichotomy, in this particular case. Also, OP never said "if you are not for Macron, you are not democratic". S/he said that Le Pen is Pro-Russia, Anti-EU and seeks to destroy that line of politics in France. That's pretty public, it's basically her plan.</t>
   </si>
   <si>
+    <t xml:space="preserve">claims about authority figures, about nazism</t>
+  </si>
+  <si>
     <t xml:space="preserve">I'm looking for an objective opinion here...is there anything about Le Pen's promises in government that isn't pandering to xenophobia? </t>
   </si>
   <si>
+    <t xml:space="preserve">care/concern about xenophobia</t>
+  </si>
+  <si>
     <t xml:space="preserve">I'm not sure if the broke any of the laws, to be honest. And by the way, back in November, Franois Hollande made a statement in which he personally, as a President, implored people to vote and support Hillary, going as far as calling Tump an imbecile. Now, that is what I call meddling, direct and impudent. Putin at least always had the decency to never express direct support over any of the candidates, and certainly never stooped to insults. In the light of Hollande's vagary, this French complains about Russia feel a bit hypocritical </t>
   </si>
   <si>
+    <t xml:space="preserve">claims about authority figures and negative actions in power</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ilhan is a fraud who supports terrorists and married her brother Edit: she also hates jews</t>
   </si>
   <si>
+    <t xml:space="preserve">concern about hating jews</t>
+  </si>
+  <si>
     <t xml:space="preserve">It's great that Satan's followers have figured out how to stop Christians forcing their religion on people. Problem is Trump doesn't give a shit about that. He is trying to rally them for the election. He wouldn't care if his actions lead to Christianity being outlawed as long as they voted for him.</t>
   </si>
   <si>
+    <t xml:space="preserve">trump and religious convincing/persecution</t>
+  </si>
+  <si>
     <t xml:space="preserve">Its not a good look for planet Earth. God bless, Macron.</t>
   </si>
   <si>
+    <t xml:space="preserve">not a good look but not sure about what</t>
+  </si>
+  <si>
     <t xml:space="preserve">Its honestly crazy to me that people justify this by saying its big corporations. Stealing is stealing, whether its something expensive, cheap, corporations, or small business. Wrong is wrong. I could see the justification if it was a steal bread to feed your family scenario, but just for the thrill of it? Yes, OP needs to seek help to see what drives this</t>
   </si>
   <si>
+    <t xml:space="preserve">expresses care about family, and concern for stealing</t>
+  </si>
+  <si>
     <t xml:space="preserve">Im a nurse, and heres how this is going to play out. Every healthcare provider that you see is going to see right through this. Theyre going to include in their report to their colleagues that youre attention seeking and theyre going to roll their eyes. Youre not fooling anyone. You dont get a pass for this. This is your way of trying to gain sympathy, and its manipulative. Its nauseating. You clearly do need help, because normal functioning people dont behave like you do. But youre not fooling a goddamn person. Good luck, asshole. Youre going to need it.</t>
   </si>
   <si>
+    <t xml:space="preserve">concern about manipulation, and normality</t>
+  </si>
+  <si>
     <t xml:space="preserve">Le pen: "I am not copying a speech made by another human being because I consider Fillon a sub-human that will be thrown into a concentration camp as soon as I'm presi..." "Erm, vive la france, freedom for all, I do not condone the murder of jewish people and/or none-whites" </t>
   </si>
   <si>
+    <t xml:space="preserve">Le Pen's statements, and also about murder</t>
+  </si>
+  <si>
     <t xml:space="preserve">Let's not exaggerate. Let's be honests with ourselves. In Romania someone like Orban or Le Pen would never rise. But not because of the welcoming tolerance and political intelligence of the Romanian people, or at least not mainly because of that. The main factor that prohibits the rise of classical populists (you may argue that PSD is populist, yes, but to a certain degree) is the much too recent memory of a hated and horrible regime. I'm talking here about the fascist type of communism we had here. </t>
   </si>
   <si>
+    <t xml:space="preserve">concern about recent authoritatian regime</t>
+  </si>
+  <si>
     <t xml:space="preserve">Most recently, that reminds of Le Pen's denial of the crimes and violations by Vichy France as not perpetrated by the French. She wants young French people to be proud of their nation, not by celebrating their achievements, but by ignoring their faults.</t>
   </si>
   <si>
+    <t xml:space="preserve">denial of crime by authority figure</t>
+  </si>
+  <si>
     <t xml:space="preserve">NTA. Your mother is an absolute asshole. To tell a small child something so horrible and untrue is psychopathic behavior. I wouldnt let this woman within screaming distance of my children ever again.</t>
   </si>
   <si>
+    <t xml:space="preserve">concern about mother's psychopathoc actions</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not all of them are a annoying and frankly shocking .... But i get what you're saying,myself i live close to a university and i can tell you i see them A LOT there.They're so god damn oppressive (VOTE Mlenchon !Don't believe the others they're terrible persons !Mlenchon is good!Mlenchon knows our issues !) These type of person just disgust me(for any candidate really)But the Mlenchon people are very present on social network too(same with Le pen people) making them believe that they're "le peuple." At this point,it's just a cult of personality.</t>
   </si>
   <si>
+    <t xml:space="preserve">disgust about political supporters</t>
+  </si>
+  <si>
     <t xml:space="preserve">Omg the fuck is wrong with these schools. What kinda of obnoxious adminstration makes shit like this.</t>
   </si>
   <si>
+    <t xml:space="preserve">anger about administration</t>
+  </si>
+  <si>
     <t xml:space="preserve">Or you could just use ratemyprofessor.com because trust me u will eventually meet a guy prof who is a asshole. Regardless of how u dress or laugh. Just use the website. It has nothing to do with you and more with them.</t>
   </si>
   <si>
+    <t xml:space="preserve">concern about bad profs</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sick of these utter degenerates. Just remove from society. They clearly have criminal intent. Physical removal.</t>
   </si>
   <si>
+    <t xml:space="preserve">disgust about "degenerates" and needing to remove them from society</t>
+  </si>
+  <si>
     <t xml:space="preserve">Still better that not even trying like macron or fillon, who are saying they care about climate change but don't actually propose to do anything meaningful about it. </t>
   </si>
   <si>
+    <t xml:space="preserve">authority figures claiming to care but in actuality don't really</t>
+  </si>
+  <si>
     <t xml:space="preserve">Supporting communism isnt the way to fix sinophobia. The CCP are literal evil, the people arent.</t>
   </si>
   <si>
+    <t xml:space="preserve">claims about sinophobia (discrimination) and about the evil of China's authority (CCP)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Thank god, a Le pen victory would have been disastrous to many people and countries, not just Muslims or France.</t>
   </si>
   <si>
+    <t xml:space="preserve">speaking of le pen's vectory</t>
+  </si>
+  <si>
     <t xml:space="preserve">The US is fascist. If you were a marginalized person youd know that to your soul. We have a fascist nazi dictator in the White House.</t>
   </si>
   <si>
+    <t xml:space="preserve">care for marginalized + criticism of authority</t>
+  </si>
+  <si>
     <t xml:space="preserve">They weren't discredited a large minority of Republican voters simply ignored the facts. Trump's a scumbag virtually nothing said about him was false. At least he wasnt a literal facist like Le Pen.</t>
   </si>
   <si>
+    <t xml:space="preserve">accusation of trump as fascist</t>
+  </si>
+  <si>
     <t xml:space="preserve">This is not some uncontrollable thing. You have a choice. Youre the kind of person who could rape someone and not take accountability. Get some fucking help</t>
   </si>
   <si>
+    <t xml:space="preserve">care for whether the person is accountable or not for sexual crime</t>
+  </si>
+  <si>
     <t xml:space="preserve">Translation: Marine le Pen is literally Hitler, and if you vote for the National Front then you're an evil racist nazi homophobe islamophobe etc etc etc... Nobody is listening to this clown.</t>
   </si>
   <si>
+    <t xml:space="preserve">discrediting an individual for expressing anti le pen remarks</t>
+  </si>
+  <si>
     <t xml:space="preserve">Trump commited crimes against humanity on Americans and therefore deserves significant criminal indictments, not prizes.</t>
   </si>
   <si>
+    <t xml:space="preserve">accusing trump, care for his crimes against humanity</t>
+  </si>
+  <si>
     <t xml:space="preserve">What you described is strictly a far-left wing issue. I don't understand why you would resort to the alt-right to search for a solution there. No far-right politician is going to fix those issues, in fact they'd inflate them greatly. If you were convinced by Le Pen that she would solve these problems, you were tricked and lied to, because it is exclusively in a right-wing politician's interest to keep doing such things in order to line their pockets. The right is full of hateful politicians with no human decency, no morals, and no truth.</t>
   </si>
   <si>
+    <t xml:space="preserve">accusing far right politicians of having no morals</t>
+  </si>
+  <si>
     <t xml:space="preserve">Wtf is wrong with these ppl? Seriously I can't understand what is actually wrong with their heads and wonder if they're like this in their normal lives. Are they some poor kids parents, do they ever laugh and have fun on the weekends, does their family know what shitty humans they are? Lol I just can't wrap my head around how there's so many heartless assholes waltzing around out there, pretending to be normal.</t>
   </si>
   <si>
+    <t xml:space="preserve">heartless but doesn't suggest why</t>
+  </si>
+  <si>
     <t xml:space="preserve">Wtf. He is a big asshole. You should leave him. Dont let him do this with you. Go to the police to get your car back. And leave. He isnt your boss. Thisis not how a relationship schould be. Do you want to do the rest of your life what he want? Imagine how it will be with a child? Imagine he decides everything, where it goes to school, what hobbies it have and dont even ask you. Only let you pay ect...</t>
   </si>
   <si>
+    <t xml:space="preserve">care for the person who is being abused</t>
+  </si>
+  <si>
     <t xml:space="preserve">YOU'RE UNDERREACTING HE'S DRUGGED YOU. HE'S GONNA DO IT AGAIN HE DOES NOT RESPECT YOUR BODILY AUTONOMY HE'S COMMITTED A CRIME AGAINST YOU</t>
   </si>
   <si>
     <t xml:space="preserve">YTA, you violated his personal and religious boundaries. Also tricking someone into drinking alchohol against their will has to be illegal.</t>
   </si>
   <si>
+    <t xml:space="preserve">accusation of lack of care of someone's boundaries and making them "impure" by alcohol</t>
+  </si>
+  <si>
     <t xml:space="preserve">YTA. This is what I've never understood about Christians. Why are yall sooooo judgemental? Doesn't God give us free will? If you wholeheartedly ask for forgiveness and mean what you say won't you be forgiven for your sins? It's her body to do what she pleases with. You are controlling over something that has nothing to do with you and it is creepy.</t>
   </si>
   <si>
+    <t xml:space="preserve">accusation of christians being too concerned with purity</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yes. You should look at the actual migration and secularism/Islam policies of all the candidates as well as their other policies; Trump for instance has some extremely dangerous policies on secularism, war, torture, the climate, and nuclear proliferation that are significantly overshadowed in the public discourse by those on Islam, and Le Pen would likely be a loyal stooge for him. Fillon or maybe even Macron could be possibilities for you.</t>
   </si>
   <si>
+    <t xml:space="preserve">concern about violence propagated by leaders</t>
+  </si>
+  <si>
     <t xml:space="preserve">Your parents are arseholes. That bullshit favouritism is disgusting. Never feel bad. Ever.</t>
   </si>
   <si>
+    <t xml:space="preserve">favoritism from parents, authority figures</t>
+  </si>
+  <si>
     <t xml:space="preserve">illegal immigration was already records low and stock market always goes up when a pro-business conservative is elected like macron. Everything else is a joke, no legislation, extreme nepotism, highly inefficient government, fighting against its own judiciary. This is just the start. Institutional corruption is no joke.</t>
   </si>
   <si>
+    <t xml:space="preserve">concern about election and corruption</t>
+  </si>
+  <si>
     <t xml:space="preserve">youre low key pretty sure? its absolutely blatantly unequivocally 100% child abuse. these parents are abusive pieces of shit who should have been sterilized and jailed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">care about child abuse, criticism of parents</t>
   </si>
 </sst>
 </file>
@@ -287,10 +404,13 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1030,13 +1150,28 @@
       <c r="D15">
         <v>1</v>
       </c>
+      <c r="H15" t="s">
+        <v>38</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="16" ht="28.5">
       <c r="A16">
         <v>4003</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="H16" t="s">
         <v>38</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="17" ht="42.75">
@@ -1044,7 +1179,16 @@
         <v>4294</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="H17" t="s">
+        <v>38</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="18" ht="42.75">
@@ -1052,7 +1196,16 @@
         <v>5101</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="H18" t="s">
+        <v>42</v>
+      </c>
+      <c r="I18" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="19">
@@ -1060,7 +1213,16 @@
         <v>6071</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="H19" t="s">
+        <v>44</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="20" ht="57">
@@ -1068,7 +1230,16 @@
         <v>6198</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="H20" t="s">
+        <v>46</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="21" ht="42.75">
@@ -1076,7 +1247,19 @@
         <v>6220</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="H21" t="s">
+        <v>48</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="22" ht="85.5">
@@ -1084,7 +1267,16 @@
         <v>6437</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="H22" t="s">
+        <v>50</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="23" ht="71.25">
@@ -1092,7 +1284,16 @@
         <v>6648</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="H23" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="24" ht="28.5">
@@ -1100,7 +1301,16 @@
         <v>6854</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>46</v>
+        <v>53</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="H24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="25" ht="85.5">
@@ -1108,7 +1318,16 @@
         <v>6890</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>47</v>
+        <v>55</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="H25" t="s">
+        <v>56</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="26">
@@ -1116,7 +1335,16 @@
         <v>7368</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="H26" t="s">
+        <v>58</v>
+      </c>
+      <c r="I26" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="27" ht="57">
@@ -1124,7 +1352,19 @@
         <v>7941</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>49</v>
+        <v>59</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="H27" t="s">
+        <v>60</v>
+      </c>
+      <c r="I27" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="28">
@@ -1132,7 +1372,16 @@
         <v>8112</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>50</v>
+        <v>61</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+      <c r="H28" t="s">
+        <v>62</v>
+      </c>
+      <c r="I28" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="29" ht="57">
@@ -1140,7 +1389,16 @@
         <v>8153</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>51</v>
+        <v>63</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="H29" t="s">
+        <v>64</v>
+      </c>
+      <c r="I29" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="30" ht="85.5">
@@ -1148,7 +1406,19 @@
         <v>8241</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>52</v>
+        <v>65</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="H30" t="s">
+        <v>66</v>
+      </c>
+      <c r="I30" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="31" ht="42.75">
@@ -1156,7 +1426,19 @@
         <v>8718</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>53</v>
+        <v>67</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <v>1</v>
+      </c>
+      <c r="H31" t="s">
+        <v>68</v>
+      </c>
+      <c r="I31" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="32" ht="85.5">
@@ -1164,7 +1446,16 @@
         <v>8771</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>54</v>
+        <v>69</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="H32" t="s">
+        <v>70</v>
+      </c>
+      <c r="I32" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="33" ht="42.75">
@@ -1172,7 +1463,16 @@
         <v>9494</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>55</v>
+        <v>71</v>
+      </c>
+      <c r="D33">
+        <v>1</v>
+      </c>
+      <c r="H33" t="s">
+        <v>72</v>
+      </c>
+      <c r="I33" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="34" ht="42.75">
@@ -1180,7 +1480,16 @@
         <v>9865</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>56</v>
+        <v>73</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="H34" t="s">
+        <v>74</v>
+      </c>
+      <c r="I34" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="35" ht="99.75">
@@ -1188,7 +1497,19 @@
         <v>10266</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>57</v>
+        <v>75</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="H35" t="s">
+        <v>76</v>
+      </c>
+      <c r="I35" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="36" ht="28.5">
@@ -1196,7 +1517,16 @@
         <v>10671</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>58</v>
+        <v>77</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="H36" t="s">
+        <v>78</v>
+      </c>
+      <c r="I36" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="37" ht="42.75">
@@ -1204,7 +1534,16 @@
         <v>10792</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>59</v>
+        <v>79</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="H37" t="s">
+        <v>80</v>
+      </c>
+      <c r="I37" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="38" ht="28.5">
@@ -1212,7 +1551,16 @@
         <v>11616</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>60</v>
+        <v>81</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="H38" t="s">
+        <v>82</v>
+      </c>
+      <c r="I38" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="39" ht="28.5">
@@ -1220,7 +1568,16 @@
         <v>12001</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>61</v>
+        <v>83</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="H39" t="s">
+        <v>84</v>
+      </c>
+      <c r="I39" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="40" ht="28.5">
@@ -1228,7 +1585,19 @@
         <v>12056</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>62</v>
+        <v>85</v>
+      </c>
+      <c r="C40">
+        <v>1</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="H40" t="s">
+        <v>86</v>
+      </c>
+      <c r="I40" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="41" ht="28.5">
@@ -1236,7 +1605,16 @@
         <v>12184</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>63</v>
+        <v>87</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="H41" t="s">
+        <v>88</v>
+      </c>
+      <c r="I41" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="42" ht="28.5">
@@ -1244,7 +1622,19 @@
         <v>12660</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>64</v>
+        <v>89</v>
+      </c>
+      <c r="C42">
+        <v>1</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="H42" t="s">
+        <v>90</v>
+      </c>
+      <c r="I42" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="43" ht="42.75">
@@ -1252,7 +1642,16 @@
         <v>13485</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>65</v>
+        <v>91</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+      <c r="H43" t="s">
+        <v>92</v>
+      </c>
+      <c r="I43" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="44" ht="28.5">
@@ -1260,7 +1659,19 @@
         <v>13699</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>66</v>
+        <v>93</v>
+      </c>
+      <c r="C44">
+        <v>1</v>
+      </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
+      <c r="H44" t="s">
+        <v>94</v>
+      </c>
+      <c r="I44" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="45" ht="28.5">
@@ -1268,7 +1679,16 @@
         <v>14088</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>67</v>
+        <v>95</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="H45" t="s">
+        <v>96</v>
+      </c>
+      <c r="I45" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="46" ht="28.5">
@@ -1276,7 +1696,19 @@
         <v>14130</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>68</v>
+        <v>97</v>
+      </c>
+      <c r="C46">
+        <v>1</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+      <c r="H46" t="s">
+        <v>98</v>
+      </c>
+      <c r="I46" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="47" ht="85.5">
@@ -1284,7 +1716,19 @@
         <v>14939</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>69</v>
+        <v>99</v>
+      </c>
+      <c r="C47">
+        <v>1</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="H47" t="s">
+        <v>100</v>
+      </c>
+      <c r="I47" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="48" ht="71.25">
@@ -1292,7 +1736,16 @@
         <v>15407</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>70</v>
+        <v>101</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="H48" t="s">
+        <v>102</v>
+      </c>
+      <c r="I48" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="49" ht="71.25">
@@ -1300,7 +1753,16 @@
         <v>15411</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>71</v>
+        <v>103</v>
+      </c>
+      <c r="C49">
+        <v>1</v>
+      </c>
+      <c r="H49" t="s">
+        <v>104</v>
+      </c>
+      <c r="I49" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="50" ht="28.5">
@@ -1308,7 +1770,16 @@
         <v>15427</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>72</v>
+        <v>105</v>
+      </c>
+      <c r="C50">
+        <v>1</v>
+      </c>
+      <c r="H50" t="s">
+        <v>104</v>
+      </c>
+      <c r="I50" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="51" ht="28.5">
@@ -1316,7 +1787,19 @@
         <v>15482</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>73</v>
+        <v>106</v>
+      </c>
+      <c r="C51">
+        <v>1</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="H51" t="s">
+        <v>107</v>
+      </c>
+      <c r="I51" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="52" ht="57">
@@ -1324,7 +1807,16 @@
         <v>15509</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>74</v>
+        <v>108</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="H52" t="s">
+        <v>109</v>
+      </c>
+      <c r="I52" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="53" ht="71.25">
@@ -1332,7 +1824,19 @@
         <v>15981</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>75</v>
+        <v>110</v>
+      </c>
+      <c r="C53">
+        <v>1</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+      <c r="H53" t="s">
+        <v>111</v>
+      </c>
+      <c r="I53" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="54">
@@ -1340,7 +1844,16 @@
         <v>16515</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>76</v>
+        <v>112</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+      <c r="H54" t="s">
+        <v>113</v>
+      </c>
+      <c r="I54" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="55" ht="57">
@@ -1348,7 +1861,19 @@
         <v>16943</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>77</v>
+        <v>114</v>
+      </c>
+      <c r="D55">
+        <v>1</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="H55" t="s">
+        <v>115</v>
+      </c>
+      <c r="I55" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="56" ht="28.5">
@@ -1356,7 +1881,19 @@
         <v>17369</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>78</v>
+        <v>116</v>
+      </c>
+      <c r="C56">
+        <v>1</v>
+      </c>
+      <c r="D56">
+        <v>1</v>
+      </c>
+      <c r="H56" t="s">
+        <v>117</v>
+      </c>
+      <c r="I56" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>